<commit_message>
Align specific health questionnaire checks
</commit_message>
<xml_diff>
--- a/docs/refactor/health_exam_result/特定健診_項目対応表.xlsx
+++ b/docs/refactor/health_exam_result/特定健診_項目対応表.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="決定事項" sheetId="1" r:id="R2ffb403984d94f70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="値の有無の判定の整理" sheetId="2" r:id="Rc271dbee7db64a80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="項目対応表" sheetId="3" r:id="R7012a127d085452c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="コード体系メモ" sheetId="4" r:id="R97ef4f84a8834b09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="省略・代替の基準" sheetId="5" r:id="R32af8b2c86eb4243"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参照元・出典一覧" sheetId="6" r:id="Rc32b874d4c024c93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="未決・確認事項" sheetId="7" r:id="R1293b39d320f452f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="決定事項" sheetId="1" r:id="R308d7d6ada70414a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="値の有無の判定の整理" sheetId="2" r:id="Rafa86809e51a40ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="項目対応表" sheetId="3" r:id="Ref5b457446fa449b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="コード体系メモ" sheetId="4" r:id="R3a19ac592cba4f26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="省略・代替の基準" sheetId="5" r:id="R05c688f0ebb04df2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参照元・出典一覧" sheetId="6" r:id="R02edabe0f352433f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="未決・確認事項" sheetId="7" r:id="Re4350a3ff71549f2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1475,7 +1475,7 @@
         <x:v>1009001005</x:v>
       </x:c>
       <x:c r="B29" s="24" t="str">
-        <x:v>飲酒</x:v>
+        <x:v>咀嚼</x:v>
       </x:c>
       <x:c r="C29" s="24" t="str">
         <x:v>問診</x:v>
@@ -1484,7 +1484,7 @@
         <x:v>40-74歳</x:v>
       </x:c>
       <x:c r="E29" s="24" t="str">
-        <x:v>必須</x:v>
+        <x:v>必須候補</x:v>
       </x:c>
       <x:c r="F29" s="24" t="str">
         <x:v>CDコードとしてVALID</x:v>
@@ -1493,14 +1493,16 @@
         <x:v>特定健診側</x:v>
       </x:c>
       <x:c r="H29" s="24" t="str">
-        <x:v>9N786000000000011</x:v>
+        <x:v>9N872000000000011</x:v>
       </x:c>
       <x:c r="I29" s="24" t="str">
         <x:v>CD</x:v>
       </x:c>
-      <x:c r="J29" s="24" t="str"/>
+      <x:c r="J29" s="24" t="str">
+        <x:v>必須扱いか情報取得時報告か確認</x:v>
+      </x:c>
       <x:c r="K29" s="24" t="str">
-        <x:v>OID 1.2.392.200119.6.24040</x:v>
+        <x:v>OID 1.2.392.200119.6.18030</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -1508,7 +1510,7 @@
         <x:v>1009001006</x:v>
       </x:c>
       <x:c r="B30" s="24" t="str">
-        <x:v>飲酒量</x:v>
+        <x:v>食べ方1(早食い等)</x:v>
       </x:c>
       <x:c r="C30" s="24" t="str">
         <x:v>問診</x:v>
@@ -1517,25 +1519,23 @@
         <x:v>40-74歳</x:v>
       </x:c>
       <x:c r="E30" s="24" t="str">
-        <x:v>条件付き/必須候補</x:v>
+        <x:v>必須</x:v>
       </x:c>
       <x:c r="F30" s="24" t="str">
-        <x:v>CO/CDコードとしてVALID</x:v>
+        <x:v>CDコードとしてVALID</x:v>
       </x:c>
       <x:c r="G30" s="24" t="str">
         <x:v>特定健診側</x:v>
       </x:c>
       <x:c r="H30" s="24" t="str">
-        <x:v>9N791000000000011</x:v>
+        <x:v>9N766000000000011</x:v>
       </x:c>
       <x:c r="I30" s="24" t="str">
-        <x:v>CO/CD</x:v>
-      </x:c>
-      <x:c r="J30" s="24" t="str">
-        <x:v>飲酒しない場合の扱い確認</x:v>
-      </x:c>
+        <x:v>CD</x:v>
+      </x:c>
+      <x:c r="J30" s="24" t="str"/>
       <x:c r="K30" s="24" t="str">
-        <x:v>OID 1.2.392.200119.6.24050</x:v>
+        <x:v>OID 1.2.392.200119.6.2004</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -1543,7 +1543,7 @@
         <x:v>1009001007</x:v>
       </x:c>
       <x:c r="B31" s="24" t="str">
-        <x:v>睡眠</x:v>
+        <x:v>食べ方2(就寝前)</x:v>
       </x:c>
       <x:c r="C31" s="24" t="str">
         <x:v>問診</x:v>
@@ -1561,7 +1561,7 @@
         <x:v>特定健診側</x:v>
       </x:c>
       <x:c r="H31" s="24" t="str">
-        <x:v>9N796000000000011</x:v>
+        <x:v>9N771000000000011</x:v>
       </x:c>
       <x:c r="I31" s="24" t="str">
         <x:v>CD</x:v>
@@ -1576,7 +1576,7 @@
         <x:v>1009001008</x:v>
       </x:c>
       <x:c r="B32" s="24" t="str">
-        <x:v>生活習慣の改善</x:v>
+        <x:v>食べ方3(間食)</x:v>
       </x:c>
       <x:c r="C32" s="24" t="str">
         <x:v>問診</x:v>
@@ -1594,31 +1594,31 @@
         <x:v>特定健診側</x:v>
       </x:c>
       <x:c r="H32" s="24" t="str">
-        <x:v>9N801000000000011</x:v>
+        <x:v>9N782000000000011</x:v>
       </x:c>
       <x:c r="I32" s="24" t="str">
         <x:v>CD</x:v>
       </x:c>
       <x:c r="J32" s="24" t="str"/>
       <x:c r="K32" s="24" t="str">
-        <x:v>OID 1.2.392.200119.6.2007</x:v>
+        <x:v>OID 1.2.392.200119.6.18040</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="24" t="str">
-        <x:v>1009101001</x:v>
+        <x:v>1009001009</x:v>
       </x:c>
       <x:c r="B33" s="24" t="str">
-        <x:v>メタボリックシンドローム判定</x:v>
+        <x:v>食習慣</x:v>
       </x:c>
       <x:c r="C33" s="24" t="str">
-        <x:v>判定</x:v>
+        <x:v>問診</x:v>
       </x:c>
       <x:c r="D33" s="24" t="str">
         <x:v>40-74歳</x:v>
       </x:c>
       <x:c r="E33" s="24" t="str">
-        <x:v>必須候補</x:v>
+        <x:v>必須</x:v>
       </x:c>
       <x:c r="F33" s="24" t="str">
         <x:v>CDコードとしてVALID</x:v>
@@ -1627,48 +1627,219 @@
         <x:v>特定健診側</x:v>
       </x:c>
       <x:c r="H33" s="24" t="str">
-        <x:v>9N501000000000011</x:v>
+        <x:v>9N781000000000011</x:v>
       </x:c>
       <x:c r="I33" s="24" t="str">
         <x:v>CD</x:v>
       </x:c>
-      <x:c r="J33" s="24" t="str">
+      <x:c r="J33" s="24" t="str"/>
+      <x:c r="K33" s="24" t="str">
+        <x:v>OID 1.2.392.200119.6.2003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="24" t="str">
+        <x:v>1009001010</x:v>
+      </x:c>
+      <x:c r="B34" s="24" t="str">
+        <x:v>飲酒</x:v>
+      </x:c>
+      <x:c r="C34" s="24" t="str">
+        <x:v>問診</x:v>
+      </x:c>
+      <x:c r="D34" s="24" t="str">
+        <x:v>40-74歳</x:v>
+      </x:c>
+      <x:c r="E34" s="24" t="str">
+        <x:v>必須</x:v>
+      </x:c>
+      <x:c r="F34" s="24" t="str">
+        <x:v>CDコードとしてVALID</x:v>
+      </x:c>
+      <x:c r="G34" s="24" t="str">
+        <x:v>特定健診側</x:v>
+      </x:c>
+      <x:c r="H34" s="24" t="str">
+        <x:v>9N786000000000011</x:v>
+      </x:c>
+      <x:c r="I34" s="24" t="str">
+        <x:v>CD</x:v>
+      </x:c>
+      <x:c r="J34" s="24" t="str"/>
+      <x:c r="K34" s="24" t="str">
+        <x:v>OID 1.2.392.200119.6.24040</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="24" t="str">
+        <x:v>1009001011</x:v>
+      </x:c>
+      <x:c r="B35" s="24" t="str">
+        <x:v>飲酒量</x:v>
+      </x:c>
+      <x:c r="C35" s="24" t="str">
+        <x:v>問診</x:v>
+      </x:c>
+      <x:c r="D35" s="24" t="str">
+        <x:v>40-74歳</x:v>
+      </x:c>
+      <x:c r="E35" s="24" t="str">
+        <x:v>条件付き/必須候補</x:v>
+      </x:c>
+      <x:c r="F35" s="24" t="str">
+        <x:v>CO/CDコードとしてVALID</x:v>
+      </x:c>
+      <x:c r="G35" s="24" t="str">
+        <x:v>特定健診側</x:v>
+      </x:c>
+      <x:c r="H35" s="24" t="str">
+        <x:v>9N791000000000011</x:v>
+      </x:c>
+      <x:c r="I35" s="24" t="str">
+        <x:v>CO/CD</x:v>
+      </x:c>
+      <x:c r="J35" s="24" t="str">
+        <x:v>飲酒しない場合の扱い確認</x:v>
+      </x:c>
+      <x:c r="K35" s="24" t="str">
+        <x:v>OID 1.2.392.200119.6.24050</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="24" t="str">
+        <x:v>1009001012</x:v>
+      </x:c>
+      <x:c r="B36" s="24" t="str">
+        <x:v>睡眠</x:v>
+      </x:c>
+      <x:c r="C36" s="24" t="str">
+        <x:v>問診</x:v>
+      </x:c>
+      <x:c r="D36" s="24" t="str">
+        <x:v>40-74歳</x:v>
+      </x:c>
+      <x:c r="E36" s="24" t="str">
+        <x:v>必須</x:v>
+      </x:c>
+      <x:c r="F36" s="24" t="str">
+        <x:v>CDコードとしてVALID</x:v>
+      </x:c>
+      <x:c r="G36" s="24" t="str">
+        <x:v>特定健診側</x:v>
+      </x:c>
+      <x:c r="H36" s="24" t="str">
+        <x:v>9N796000000000011</x:v>
+      </x:c>
+      <x:c r="I36" s="24" t="str">
+        <x:v>CD</x:v>
+      </x:c>
+      <x:c r="J36" s="24" t="str"/>
+      <x:c r="K36" s="24" t="str">
+        <x:v>OID 1.2.392.200119.6.2003</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="24" t="str">
+        <x:v>1009001013</x:v>
+      </x:c>
+      <x:c r="B37" s="24" t="str">
+        <x:v>生活習慣の改善</x:v>
+      </x:c>
+      <x:c r="C37" s="24" t="str">
+        <x:v>問診</x:v>
+      </x:c>
+      <x:c r="D37" s="24" t="str">
+        <x:v>40-74歳</x:v>
+      </x:c>
+      <x:c r="E37" s="24" t="str">
+        <x:v>必須</x:v>
+      </x:c>
+      <x:c r="F37" s="24" t="str">
+        <x:v>CDコードとしてVALID</x:v>
+      </x:c>
+      <x:c r="G37" s="24" t="str">
+        <x:v>特定健診側</x:v>
+      </x:c>
+      <x:c r="H37" s="24" t="str">
+        <x:v>9N801000000000011</x:v>
+      </x:c>
+      <x:c r="I37" s="24" t="str">
+        <x:v>CD</x:v>
+      </x:c>
+      <x:c r="J37" s="24" t="str"/>
+      <x:c r="K37" s="24" t="str">
+        <x:v>OID 1.2.392.200119.6.2007</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="24" t="str">
+        <x:v>1009101001</x:v>
+      </x:c>
+      <x:c r="B38" s="24" t="str">
+        <x:v>メタボリックシンドローム判定</x:v>
+      </x:c>
+      <x:c r="C38" s="24" t="str">
+        <x:v>判定</x:v>
+      </x:c>
+      <x:c r="D38" s="24" t="str">
+        <x:v>40-74歳</x:v>
+      </x:c>
+      <x:c r="E38" s="24" t="str">
+        <x:v>必須候補</x:v>
+      </x:c>
+      <x:c r="F38" s="24" t="str">
+        <x:v>CDコードとしてVALID</x:v>
+      </x:c>
+      <x:c r="G38" s="24" t="str">
+        <x:v>特定健診側</x:v>
+      </x:c>
+      <x:c r="H38" s="24" t="str">
+        <x:v>9N501000000000011</x:v>
+      </x:c>
+      <x:c r="I38" s="24" t="str">
+        <x:v>CD</x:v>
+      </x:c>
+      <x:c r="J38" s="24" t="str">
         <x:v>医師の診断とは別。必須扱いの再確認</x:v>
       </x:c>
-      <x:c r="K33" s="24" t="str"/>
-    </x:row>
-    <x:row r="34">
-      <x:c r="A34" s="21" t="str">
+      <x:c r="K38" s="24" t="str">
+        <x:v>result_code_oid 1.2.392.200119.6.1008</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="21" t="str">
         <x:v>1009101002</x:v>
       </x:c>
-      <x:c r="B34" s="21" t="str">
+      <x:c r="B39" s="21" t="str">
         <x:v>保健指導レベル</x:v>
       </x:c>
-      <x:c r="C34" s="21" t="str">
+      <x:c r="C39" s="21" t="str">
         <x:v>判定</x:v>
       </x:c>
-      <x:c r="D34" s="21" t="str">
+      <x:c r="D39" s="21" t="str">
         <x:v>40-74歳</x:v>
       </x:c>
-      <x:c r="E34" s="21" t="str">
+      <x:c r="E39" s="21" t="str">
         <x:v>必須候補</x:v>
       </x:c>
-      <x:c r="F34" s="21" t="str">
+      <x:c r="F39" s="21" t="str">
         <x:v>CDコードとしてVALID</x:v>
       </x:c>
-      <x:c r="G34" s="21" t="str">
+      <x:c r="G39" s="21" t="str">
         <x:v>特定健診側</x:v>
       </x:c>
-      <x:c r="H34" s="21" t="str">
+      <x:c r="H39" s="21" t="str">
         <x:v>9N506000000000011</x:v>
       </x:c>
-      <x:c r="I34" s="21" t="str">
+      <x:c r="I39" s="21" t="str">
         <x:v>CD</x:v>
       </x:c>
-      <x:c r="J34" s="21" t="str">
+      <x:c r="J39" s="21" t="str">
         <x:v>必須扱いの再確認</x:v>
       </x:c>
-      <x:c r="K34" s="21" t="str"/>
+      <x:c r="K39" s="21" t="str">
+        <x:v>result_code_oid 1.2.392.200119.6.3001</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3003,10 +3174,10 @@
         <x:v>1009001005</x:v>
       </x:c>
       <x:c r="B55" s="24" t="str">
-        <x:v>飲酒</x:v>
+        <x:v>咀嚼</x:v>
       </x:c>
       <x:c r="C55" s="24" t="str">
-        <x:v>9N786000000000011</x:v>
+        <x:v>9N872000000000011</x:v>
       </x:c>
       <x:c r="D55" s="24" t="str"/>
       <x:c r="E55" s="24" t="str">
@@ -3020,7 +3191,7 @@
         <x:v>候補</x:v>
       </x:c>
       <x:c r="I55" s="24" t="str">
-        <x:v>OID 1.2.392.200119.6.24040</x:v>
+        <x:v>必須扱いか情報取得時報告か確認</x:v>
       </x:c>
       <x:c r="J55" s="21"/>
     </x:row>
@@ -3029,14 +3200,14 @@
         <x:v>1009001006</x:v>
       </x:c>
       <x:c r="B56" s="24" t="str">
-        <x:v>飲酒量</x:v>
+        <x:v>食べ方1(早食い等)</x:v>
       </x:c>
       <x:c r="C56" s="24" t="str">
-        <x:v>9N791000000000011</x:v>
+        <x:v>9N766000000000011</x:v>
       </x:c>
       <x:c r="D56" s="24" t="str"/>
       <x:c r="E56" s="24" t="str">
-        <x:v>CO/CD</x:v>
+        <x:v>CD</x:v>
       </x:c>
       <x:c r="F56" s="24" t="str">
         <x:v>RESULT_VALUE</x:v>
@@ -3046,7 +3217,7 @@
         <x:v>候補</x:v>
       </x:c>
       <x:c r="I56" s="24" t="str">
-        <x:v>飲酒しない場合の扱い確認</x:v>
+        <x:v>OID 1.2.392.200119.6.2004</x:v>
       </x:c>
       <x:c r="J56" s="21"/>
     </x:row>
@@ -3055,10 +3226,10 @@
         <x:v>1009001007</x:v>
       </x:c>
       <x:c r="B57" s="24" t="str">
-        <x:v>睡眠</x:v>
+        <x:v>食べ方2(就寝前)</x:v>
       </x:c>
       <x:c r="C57" s="24" t="str">
-        <x:v>9N796000000000011</x:v>
+        <x:v>9N771000000000011</x:v>
       </x:c>
       <x:c r="D57" s="24" t="str"/>
       <x:c r="E57" s="24" t="str">
@@ -3081,10 +3252,10 @@
         <x:v>1009001008</x:v>
       </x:c>
       <x:c r="B58" s="24" t="str">
-        <x:v>生活習慣の改善</x:v>
+        <x:v>食べ方3(間食)</x:v>
       </x:c>
       <x:c r="C58" s="24" t="str">
-        <x:v>9N801000000000011</x:v>
+        <x:v>9N782000000000011</x:v>
       </x:c>
       <x:c r="D58" s="24" t="str"/>
       <x:c r="E58" s="24" t="str">
@@ -3098,19 +3269,19 @@
         <x:v>候補</x:v>
       </x:c>
       <x:c r="I58" s="24" t="str">
-        <x:v>OID 1.2.392.200119.6.2007</x:v>
+        <x:v>OID 1.2.392.200119.6.18040</x:v>
       </x:c>
       <x:c r="J58" s="21"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="24" t="str">
-        <x:v>1009101001</x:v>
+        <x:v>1009001009</x:v>
       </x:c>
       <x:c r="B59" s="24" t="str">
-        <x:v>メタボリックシンドローム判定</x:v>
+        <x:v>食習慣</x:v>
       </x:c>
       <x:c r="C59" s="24" t="str">
-        <x:v>9N501000000000011</x:v>
+        <x:v>9N781000000000011</x:v>
       </x:c>
       <x:c r="D59" s="24" t="str"/>
       <x:c r="E59" s="24" t="str">
@@ -3124,35 +3295,165 @@
         <x:v>候補</x:v>
       </x:c>
       <x:c r="I59" s="24" t="str">
+        <x:v>OID 1.2.392.200119.6.2003</x:v>
+      </x:c>
+      <x:c r="J59" s="21"/>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="24" t="str">
+        <x:v>1009001010</x:v>
+      </x:c>
+      <x:c r="B60" s="24" t="str">
+        <x:v>飲酒</x:v>
+      </x:c>
+      <x:c r="C60" s="24" t="str">
+        <x:v>9N786000000000011</x:v>
+      </x:c>
+      <x:c r="D60" s="24" t="str"/>
+      <x:c r="E60" s="24" t="str">
+        <x:v>CD</x:v>
+      </x:c>
+      <x:c r="F60" s="24" t="str">
+        <x:v>RESULT_VALUE</x:v>
+      </x:c>
+      <x:c r="G60" s="24" t="str"/>
+      <x:c r="H60" s="24" t="str">
+        <x:v>候補</x:v>
+      </x:c>
+      <x:c r="I60" s="24" t="str">
+        <x:v>OID 1.2.392.200119.6.24040</x:v>
+      </x:c>
+      <x:c r="J60" s="21"/>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="24" t="str">
+        <x:v>1009001011</x:v>
+      </x:c>
+      <x:c r="B61" s="24" t="str">
+        <x:v>飲酒量</x:v>
+      </x:c>
+      <x:c r="C61" s="24" t="str">
+        <x:v>9N791000000000011</x:v>
+      </x:c>
+      <x:c r="D61" s="24" t="str"/>
+      <x:c r="E61" s="24" t="str">
+        <x:v>CO/CD</x:v>
+      </x:c>
+      <x:c r="F61" s="24" t="str">
+        <x:v>RESULT_VALUE</x:v>
+      </x:c>
+      <x:c r="G61" s="24" t="str"/>
+      <x:c r="H61" s="24" t="str">
+        <x:v>候補</x:v>
+      </x:c>
+      <x:c r="I61" s="24" t="str">
+        <x:v>飲酒しない場合の扱い確認</x:v>
+      </x:c>
+      <x:c r="J61" s="21"/>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="24" t="str">
+        <x:v>1009001012</x:v>
+      </x:c>
+      <x:c r="B62" s="24" t="str">
+        <x:v>睡眠</x:v>
+      </x:c>
+      <x:c r="C62" s="24" t="str">
+        <x:v>9N796000000000011</x:v>
+      </x:c>
+      <x:c r="D62" s="24" t="str"/>
+      <x:c r="E62" s="24" t="str">
+        <x:v>CD</x:v>
+      </x:c>
+      <x:c r="F62" s="24" t="str">
+        <x:v>RESULT_VALUE</x:v>
+      </x:c>
+      <x:c r="G62" s="24" t="str"/>
+      <x:c r="H62" s="24" t="str">
+        <x:v>候補</x:v>
+      </x:c>
+      <x:c r="I62" s="24" t="str">
+        <x:v>OID 1.2.392.200119.6.2003</x:v>
+      </x:c>
+      <x:c r="J62" s="21"/>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="24" t="str">
+        <x:v>1009001013</x:v>
+      </x:c>
+      <x:c r="B63" s="24" t="str">
+        <x:v>生活習慣の改善</x:v>
+      </x:c>
+      <x:c r="C63" s="24" t="str">
+        <x:v>9N801000000000011</x:v>
+      </x:c>
+      <x:c r="D63" s="24" t="str"/>
+      <x:c r="E63" s="24" t="str">
+        <x:v>CD</x:v>
+      </x:c>
+      <x:c r="F63" s="24" t="str">
+        <x:v>RESULT_VALUE</x:v>
+      </x:c>
+      <x:c r="G63" s="24" t="str"/>
+      <x:c r="H63" s="24" t="str">
+        <x:v>候補</x:v>
+      </x:c>
+      <x:c r="I63" s="24" t="str">
+        <x:v>OID 1.2.392.200119.6.2007</x:v>
+      </x:c>
+      <x:c r="J63" s="21"/>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" s="24" t="str">
+        <x:v>1009101001</x:v>
+      </x:c>
+      <x:c r="B64" s="24" t="str">
+        <x:v>メタボリックシンドローム判定</x:v>
+      </x:c>
+      <x:c r="C64" s="24" t="str">
+        <x:v>9N501000000000011</x:v>
+      </x:c>
+      <x:c r="D64" s="24" t="str"/>
+      <x:c r="E64" s="24" t="str">
+        <x:v>CD</x:v>
+      </x:c>
+      <x:c r="F64" s="24" t="str">
+        <x:v>RESULT_VALUE</x:v>
+      </x:c>
+      <x:c r="G64" s="24" t="str"/>
+      <x:c r="H64" s="24" t="str">
+        <x:v>候補</x:v>
+      </x:c>
+      <x:c r="I64" s="24" t="str">
         <x:v>医師の診断とは別。必須扱いの再確認</x:v>
       </x:c>
-      <x:c r="J59" s="21"/>
-    </x:row>
-    <x:row r="60">
-      <x:c r="A60" s="21" t="str">
+      <x:c r="J64" s="21"/>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="21" t="str">
         <x:v>1009101002</x:v>
       </x:c>
-      <x:c r="B60" s="21" t="str">
+      <x:c r="B65" s="21" t="str">
         <x:v>保健指導レベル</x:v>
       </x:c>
-      <x:c r="C60" s="21" t="str">
+      <x:c r="C65" s="21" t="str">
         <x:v>9N506000000000011</x:v>
       </x:c>
-      <x:c r="D60" s="21" t="str"/>
-      <x:c r="E60" s="21" t="str">
+      <x:c r="D65" s="21" t="str"/>
+      <x:c r="E65" s="21" t="str">
         <x:v>CD</x:v>
       </x:c>
-      <x:c r="F60" s="21" t="str">
-        <x:v>RESULT_VALUE</x:v>
-      </x:c>
-      <x:c r="G60" s="21" t="str"/>
-      <x:c r="H60" s="21" t="str">
-        <x:v>候補</x:v>
-      </x:c>
-      <x:c r="I60" s="21" t="str">
+      <x:c r="F65" s="21" t="str">
+        <x:v>RESULT_VALUE</x:v>
+      </x:c>
+      <x:c r="G65" s="21" t="str"/>
+      <x:c r="H65" s="21" t="str">
+        <x:v>候補</x:v>
+      </x:c>
+      <x:c r="I65" s="21" t="str">
         <x:v>必須扱いの再確認</x:v>
       </x:c>
-      <x:c r="J60" s="21"/>
+      <x:c r="J65" s="21"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3282,19 +3583,19 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="24" t="str">
-        <x:v>1.2.392.200119.6.24040</x:v>
+        <x:v>1.2.392.200119.6.2004</x:v>
       </x:c>
       <x:c r="B7" s="24" t="str">
-        <x:v>飲酒習慣</x:v>
+        <x:v>食事の速さコード</x:v>
       </x:c>
       <x:c r="C7" s="24" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D7" s="24" t="str">
-        <x:v>毎日</x:v>
+        <x:v>速い</x:v>
       </x:c>
       <x:c r="E7" s="24" t="str">
-        <x:v>飲酒</x:v>
+        <x:v>食べ方1(早食い等)</x:v>
       </x:c>
       <x:c r="F7" s="21"/>
       <x:c r="G7" s="21"/>
@@ -3304,19 +3605,19 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="24" t="str">
-        <x:v>1.2.392.200119.6.24040</x:v>
+        <x:v>1.2.392.200119.6.2004</x:v>
       </x:c>
       <x:c r="B8" s="24" t="str">
-        <x:v>飲酒習慣</x:v>
+        <x:v>食事の速さコード</x:v>
       </x:c>
       <x:c r="C8" s="24" t="str">
         <x:v>2</x:v>
       </x:c>
       <x:c r="D8" s="24" t="str">
-        <x:v>週5~6日</x:v>
+        <x:v>ふつう</x:v>
       </x:c>
       <x:c r="E8" s="24" t="str">
-        <x:v>飲酒</x:v>
+        <x:v>食べ方1(早食い等)</x:v>
       </x:c>
       <x:c r="F8" s="21"/>
       <x:c r="G8" s="21"/>
@@ -3326,19 +3627,19 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="24" t="str">
-        <x:v>1.2.392.200119.6.24040</x:v>
+        <x:v>1.2.392.200119.6.2004</x:v>
       </x:c>
       <x:c r="B9" s="24" t="str">
-        <x:v>飲酒習慣</x:v>
+        <x:v>食事の速さコード</x:v>
       </x:c>
       <x:c r="C9" s="24" t="str">
         <x:v>3</x:v>
       </x:c>
       <x:c r="D9" s="24" t="str">
-        <x:v>週に3~4日</x:v>
+        <x:v>遅い</x:v>
       </x:c>
       <x:c r="E9" s="24" t="str">
-        <x:v>飲酒</x:v>
+        <x:v>食べ方1(早食い等)</x:v>
       </x:c>
       <x:c r="F9" s="21"/>
       <x:c r="G9" s="21"/>
@@ -3354,10 +3655,10 @@
         <x:v>飲酒習慣</x:v>
       </x:c>
       <x:c r="C10" s="24" t="str">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D10" s="24" t="str">
-        <x:v>週に1~2日</x:v>
+        <x:v>毎日</x:v>
       </x:c>
       <x:c r="E10" s="24" t="str">
         <x:v>飲酒</x:v>
@@ -3376,10 +3677,10 @@
         <x:v>飲酒習慣</x:v>
       </x:c>
       <x:c r="C11" s="24" t="str">
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D11" s="24" t="str">
-        <x:v>月に1~3日</x:v>
+        <x:v>週5~6日</x:v>
       </x:c>
       <x:c r="E11" s="24" t="str">
         <x:v>飲酒</x:v>
@@ -3398,10 +3699,10 @@
         <x:v>飲酒習慣</x:v>
       </x:c>
       <x:c r="C12" s="24" t="str">
-        <x:v>6</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D12" s="24" t="str">
-        <x:v>月に1日未満</x:v>
+        <x:v>週に3~4日</x:v>
       </x:c>
       <x:c r="E12" s="24" t="str">
         <x:v>飲酒</x:v>
@@ -3420,10 +3721,10 @@
         <x:v>飲酒習慣</x:v>
       </x:c>
       <x:c r="C13" s="24" t="str">
-        <x:v>7</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D13" s="24" t="str">
-        <x:v>やめた</x:v>
+        <x:v>週に1~2日</x:v>
       </x:c>
       <x:c r="E13" s="24" t="str">
         <x:v>飲酒</x:v>
@@ -3442,10 +3743,10 @@
         <x:v>飲酒習慣</x:v>
       </x:c>
       <x:c r="C14" s="24" t="str">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D14" s="24" t="str">
-        <x:v>飲まない(飲めない)</x:v>
+        <x:v>月に1~3日</x:v>
       </x:c>
       <x:c r="E14" s="24" t="str">
         <x:v>飲酒</x:v>
@@ -3458,19 +3759,19 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="24" t="str">
-        <x:v>1.2.392.200119.6.24050</x:v>
+        <x:v>1.2.392.200119.6.24040</x:v>
       </x:c>
       <x:c r="B15" s="24" t="str">
-        <x:v>飲酒量区分</x:v>
+        <x:v>飲酒習慣</x:v>
       </x:c>
       <x:c r="C15" s="24" t="str">
-        <x:v>1</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D15" s="24" t="str">
-        <x:v>1合未満</x:v>
+        <x:v>月に1日未満</x:v>
       </x:c>
       <x:c r="E15" s="24" t="str">
-        <x:v>飲酒量</x:v>
+        <x:v>飲酒</x:v>
       </x:c>
       <x:c r="F15" s="21"/>
       <x:c r="G15" s="21"/>
@@ -3480,19 +3781,19 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="24" t="str">
-        <x:v>1.2.392.200119.6.24050</x:v>
+        <x:v>1.2.392.200119.6.24040</x:v>
       </x:c>
       <x:c r="B16" s="24" t="str">
-        <x:v>飲酒量区分</x:v>
+        <x:v>飲酒習慣</x:v>
       </x:c>
       <x:c r="C16" s="24" t="str">
-        <x:v>2</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D16" s="24" t="str">
-        <x:v>1~2合未満</x:v>
+        <x:v>やめた</x:v>
       </x:c>
       <x:c r="E16" s="24" t="str">
-        <x:v>飲酒量</x:v>
+        <x:v>飲酒</x:v>
       </x:c>
       <x:c r="F16" s="21"/>
       <x:c r="G16" s="21"/>
@@ -3502,19 +3803,19 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="24" t="str">
-        <x:v>1.2.392.200119.6.24050</x:v>
+        <x:v>1.2.392.200119.6.24040</x:v>
       </x:c>
       <x:c r="B17" s="24" t="str">
-        <x:v>飲酒量区分</x:v>
+        <x:v>飲酒習慣</x:v>
       </x:c>
       <x:c r="C17" s="24" t="str">
-        <x:v>3</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D17" s="24" t="str">
-        <x:v>2~3合未満</x:v>
+        <x:v>飲まない(飲めない)</x:v>
       </x:c>
       <x:c r="E17" s="24" t="str">
-        <x:v>飲酒量</x:v>
+        <x:v>飲酒</x:v>
       </x:c>
       <x:c r="F17" s="21"/>
       <x:c r="G17" s="21"/>
@@ -3530,10 +3831,10 @@
         <x:v>飲酒量区分</x:v>
       </x:c>
       <x:c r="C18" s="24" t="str">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D18" s="24" t="str">
-        <x:v>3~5合未満</x:v>
+        <x:v>1合未満</x:v>
       </x:c>
       <x:c r="E18" s="24" t="str">
         <x:v>飲酒量</x:v>
@@ -3552,10 +3853,10 @@
         <x:v>飲酒量区分</x:v>
       </x:c>
       <x:c r="C19" s="24" t="str">
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D19" s="24" t="str">
-        <x:v>5合以上</x:v>
+        <x:v>1~2合未満</x:v>
       </x:c>
       <x:c r="E19" s="24" t="str">
         <x:v>飲酒量</x:v>
@@ -3568,19 +3869,19 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="24" t="str">
-        <x:v>1.2.392.200119.6.24060</x:v>
+        <x:v>1.2.392.200119.6.24050</x:v>
       </x:c>
       <x:c r="B20" s="24" t="str">
-        <x:v>喫煙</x:v>
+        <x:v>飲酒量区分</x:v>
       </x:c>
       <x:c r="C20" s="24" t="str">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D20" s="24" t="str">
-        <x:v>はい</x:v>
+        <x:v>2~3合未満</x:v>
       </x:c>
       <x:c r="E20" s="24" t="str">
-        <x:v>喫煙</x:v>
+        <x:v>飲酒量</x:v>
       </x:c>
       <x:c r="F20" s="21"/>
       <x:c r="G20" s="21"/>
@@ -3590,19 +3891,19 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="24" t="str">
-        <x:v>1.2.392.200119.6.24060</x:v>
+        <x:v>1.2.392.200119.6.24050</x:v>
       </x:c>
       <x:c r="B21" s="24" t="str">
-        <x:v>喫煙</x:v>
+        <x:v>飲酒量区分</x:v>
       </x:c>
       <x:c r="C21" s="24" t="str">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D21" s="24" t="str">
-        <x:v>以前は吸っていたが、最近1ヶ月間は吸っていない</x:v>
+        <x:v>3~5合未満</x:v>
       </x:c>
       <x:c r="E21" s="24" t="str">
-        <x:v>喫煙</x:v>
+        <x:v>飲酒量</x:v>
       </x:c>
       <x:c r="F21" s="21"/>
       <x:c r="G21" s="21"/>
@@ -3612,19 +3913,19 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="24" t="str">
-        <x:v>1.2.392.200119.6.24060</x:v>
+        <x:v>1.2.392.200119.6.24050</x:v>
       </x:c>
       <x:c r="B22" s="24" t="str">
-        <x:v>喫煙</x:v>
+        <x:v>飲酒量区分</x:v>
       </x:c>
       <x:c r="C22" s="24" t="str">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D22" s="24" t="str">
-        <x:v>いいえ</x:v>
+        <x:v>5合以上</x:v>
       </x:c>
       <x:c r="E22" s="24" t="str">
-        <x:v>喫煙</x:v>
+        <x:v>飲酒量</x:v>
       </x:c>
       <x:c r="F22" s="21"/>
       <x:c r="G22" s="21"/>
@@ -3634,19 +3935,19 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="24" t="str">
-        <x:v>1.2.392.200119.6.2007</x:v>
+        <x:v>1.2.392.200119.6.24060</x:v>
       </x:c>
       <x:c r="B23" s="24" t="str">
-        <x:v>生活習慣改善意志区分</x:v>
+        <x:v>喫煙</x:v>
       </x:c>
       <x:c r="C23" s="24" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D23" s="24" t="str">
-        <x:v>意志なし</x:v>
+        <x:v>はい</x:v>
       </x:c>
       <x:c r="E23" s="24" t="str">
-        <x:v>生活習慣の改善</x:v>
+        <x:v>喫煙</x:v>
       </x:c>
       <x:c r="F23" s="21"/>
       <x:c r="G23" s="21"/>
@@ -3656,19 +3957,19 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="24" t="str">
-        <x:v>1.2.392.200119.6.2007</x:v>
+        <x:v>1.2.392.200119.6.24060</x:v>
       </x:c>
       <x:c r="B24" s="24" t="str">
-        <x:v>生活習慣改善意志区分</x:v>
+        <x:v>喫煙</x:v>
       </x:c>
       <x:c r="C24" s="24" t="str">
         <x:v>2</x:v>
       </x:c>
       <x:c r="D24" s="24" t="str">
-        <x:v>意志あり(6ヵ月以内)</x:v>
+        <x:v>以前は吸っていたが、最近1ヶ月間は吸っていない</x:v>
       </x:c>
       <x:c r="E24" s="24" t="str">
-        <x:v>生活習慣の改善</x:v>
+        <x:v>喫煙</x:v>
       </x:c>
       <x:c r="F24" s="21"/>
       <x:c r="G24" s="21"/>
@@ -3678,19 +3979,19 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="24" t="str">
-        <x:v>1.2.392.200119.6.2007</x:v>
+        <x:v>1.2.392.200119.6.24060</x:v>
       </x:c>
       <x:c r="B25" s="24" t="str">
-        <x:v>生活習慣改善意志区分</x:v>
+        <x:v>喫煙</x:v>
       </x:c>
       <x:c r="C25" s="24" t="str">
         <x:v>3</x:v>
       </x:c>
       <x:c r="D25" s="24" t="str">
-        <x:v>意志あり(近いうち)</x:v>
+        <x:v>いいえ</x:v>
       </x:c>
       <x:c r="E25" s="24" t="str">
-        <x:v>生活習慣の改善</x:v>
+        <x:v>喫煙</x:v>
       </x:c>
       <x:c r="F25" s="21"/>
       <x:c r="G25" s="21"/>
@@ -3706,10 +4007,10 @@
         <x:v>生活習慣改善意志区分</x:v>
       </x:c>
       <x:c r="C26" s="24" t="str">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D26" s="24" t="str">
-        <x:v>取組済み(6ヵ月未満)</x:v>
+        <x:v>意志なし</x:v>
       </x:c>
       <x:c r="E26" s="24" t="str">
         <x:v>生活習慣の改善</x:v>
@@ -3728,10 +4029,10 @@
         <x:v>生活習慣改善意志区分</x:v>
       </x:c>
       <x:c r="C27" s="24" t="str">
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D27" s="24" t="str">
-        <x:v>取組済み(6ヵ月以上)</x:v>
+        <x:v>意志あり(6ヵ月以内)</x:v>
       </x:c>
       <x:c r="E27" s="24" t="str">
         <x:v>生活習慣の改善</x:v>
@@ -3744,25 +4045,267 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="24" t="str">
-        <x:v>1.2.392.200119.6.2100</x:v>
+        <x:v>1.2.392.200119.6.2007</x:v>
       </x:c>
       <x:c r="B28" s="24" t="str">
-        <x:v>陰性陽性</x:v>
+        <x:v>生活習慣改善意志区分</x:v>
       </x:c>
       <x:c r="C28" s="24" t="str">
-        <x:v>1/2等</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D28" s="24" t="str">
-        <x:v>陰性/陽性等</x:v>
+        <x:v>意志あり(近いうち)</x:v>
       </x:c>
       <x:c r="E28" s="24" t="str">
-        <x:v>便潜血など。項目ごとの正式表示は要確認</x:v>
+        <x:v>生活習慣の改善</x:v>
       </x:c>
       <x:c r="F28" s="21"/>
       <x:c r="G28" s="21"/>
       <x:c r="H28" s="21"/>
       <x:c r="I28" s="21"/>
       <x:c r="J28" s="21"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="24" t="str">
+        <x:v>1.2.392.200119.6.2007</x:v>
+      </x:c>
+      <x:c r="B29" s="24" t="str">
+        <x:v>生活習慣改善意志区分</x:v>
+      </x:c>
+      <x:c r="C29" s="24" t="str">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D29" s="24" t="str">
+        <x:v>取組済み(6ヵ月未満)</x:v>
+      </x:c>
+      <x:c r="E29" s="24" t="str">
+        <x:v>生活習慣の改善</x:v>
+      </x:c>
+      <x:c r="F29" s="21"/>
+      <x:c r="G29" s="21"/>
+      <x:c r="H29" s="21"/>
+      <x:c r="I29" s="21"/>
+      <x:c r="J29" s="21"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="24" t="str">
+        <x:v>1.2.392.200119.6.2007</x:v>
+      </x:c>
+      <x:c r="B30" s="24" t="str">
+        <x:v>生活習慣改善意志区分</x:v>
+      </x:c>
+      <x:c r="C30" s="24" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D30" s="24" t="str">
+        <x:v>取組済み(6ヵ月以上)</x:v>
+      </x:c>
+      <x:c r="E30" s="24" t="str">
+        <x:v>生活習慣の改善</x:v>
+      </x:c>
+      <x:c r="F30" s="21"/>
+      <x:c r="G30" s="21"/>
+      <x:c r="H30" s="21"/>
+      <x:c r="I30" s="21"/>
+      <x:c r="J30" s="21"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="24" t="str">
+        <x:v>1.2.392.200119.6.18030</x:v>
+      </x:c>
+      <x:c r="B31" s="24" t="str">
+        <x:v>咀嚼コード</x:v>
+      </x:c>
+      <x:c r="C31" s="24" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D31" s="24" t="str">
+        <x:v>何でも</x:v>
+      </x:c>
+      <x:c r="E31" s="24" t="str">
+        <x:v>咀嚼</x:v>
+      </x:c>
+      <x:c r="F31" s="21"/>
+      <x:c r="G31" s="21"/>
+      <x:c r="H31" s="21"/>
+      <x:c r="I31" s="21"/>
+      <x:c r="J31" s="21"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="24" t="str">
+        <x:v>1.2.392.200119.6.18030</x:v>
+      </x:c>
+      <x:c r="B32" s="24" t="str">
+        <x:v>咀嚼コード</x:v>
+      </x:c>
+      <x:c r="C32" s="24" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D32" s="24" t="str">
+        <x:v>かみにくい</x:v>
+      </x:c>
+      <x:c r="E32" s="24" t="str">
+        <x:v>咀嚼</x:v>
+      </x:c>
+      <x:c r="F32" s="21"/>
+      <x:c r="G32" s="21"/>
+      <x:c r="H32" s="21"/>
+      <x:c r="I32" s="21"/>
+      <x:c r="J32" s="21"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="24" t="str">
+        <x:v>1.2.392.200119.6.18030</x:v>
+      </x:c>
+      <x:c r="B33" s="24" t="str">
+        <x:v>咀嚼コード</x:v>
+      </x:c>
+      <x:c r="C33" s="24" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D33" s="24" t="str">
+        <x:v>ほとんどかめない</x:v>
+      </x:c>
+      <x:c r="E33" s="24" t="str">
+        <x:v>咀嚼</x:v>
+      </x:c>
+      <x:c r="F33" s="21"/>
+      <x:c r="G33" s="21"/>
+      <x:c r="H33" s="21"/>
+      <x:c r="I33" s="21"/>
+      <x:c r="J33" s="21"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="24" t="str">
+        <x:v>1.2.392.200119.6.18040</x:v>
+      </x:c>
+      <x:c r="B34" s="24" t="str">
+        <x:v>間食コード</x:v>
+      </x:c>
+      <x:c r="C34" s="24" t="str">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D34" s="24" t="str">
+        <x:v>毎日</x:v>
+      </x:c>
+      <x:c r="E34" s="24" t="str">
+        <x:v>食べ方3(間食)</x:v>
+      </x:c>
+      <x:c r="F34" s="21"/>
+      <x:c r="G34" s="21"/>
+      <x:c r="H34" s="21"/>
+      <x:c r="I34" s="21"/>
+      <x:c r="J34" s="21"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="24" t="str">
+        <x:v>1.2.392.200119.6.18040</x:v>
+      </x:c>
+      <x:c r="B35" s="24" t="str">
+        <x:v>間食コード</x:v>
+      </x:c>
+      <x:c r="C35" s="24" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D35" s="24" t="str">
+        <x:v>時々</x:v>
+      </x:c>
+      <x:c r="E35" s="24" t="str">
+        <x:v>食べ方3(間食)</x:v>
+      </x:c>
+      <x:c r="F35" s="21"/>
+      <x:c r="G35" s="21"/>
+      <x:c r="H35" s="21"/>
+      <x:c r="I35" s="21"/>
+      <x:c r="J35" s="21"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="24" t="str">
+        <x:v>1.2.392.200119.6.18040</x:v>
+      </x:c>
+      <x:c r="B36" s="24" t="str">
+        <x:v>間食コード</x:v>
+      </x:c>
+      <x:c r="C36" s="24" t="str">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D36" s="24" t="str">
+        <x:v>ほとんど摂取しない</x:v>
+      </x:c>
+      <x:c r="E36" s="24" t="str">
+        <x:v>食べ方3(間食)</x:v>
+      </x:c>
+      <x:c r="F36" s="21"/>
+      <x:c r="G36" s="21"/>
+      <x:c r="H36" s="21"/>
+      <x:c r="I36" s="21"/>
+      <x:c r="J36" s="21"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="24" t="str">
+        <x:v>1.2.392.200119.6.1008</x:v>
+      </x:c>
+      <x:c r="B37" s="24" t="str">
+        <x:v>メタボリックシンドローム判定</x:v>
+      </x:c>
+      <x:c r="C37" s="24" t="str">
+        <x:v>要確認</x:v>
+      </x:c>
+      <x:c r="D37" s="24" t="str">
+        <x:v>要確認</x:v>
+      </x:c>
+      <x:c r="E37" s="24" t="str">
+        <x:v>9N501。付属2/exam_item_masterでOID確認済み、コード値一覧は別途確認</x:v>
+      </x:c>
+      <x:c r="F37" s="21"/>
+      <x:c r="G37" s="21"/>
+      <x:c r="H37" s="21"/>
+      <x:c r="I37" s="21"/>
+      <x:c r="J37" s="21"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="24" t="str">
+        <x:v>1.2.392.200119.6.3001</x:v>
+      </x:c>
+      <x:c r="B38" s="24" t="str">
+        <x:v>保健指導レベル</x:v>
+      </x:c>
+      <x:c r="C38" s="24" t="str">
+        <x:v>要確認</x:v>
+      </x:c>
+      <x:c r="D38" s="24" t="str">
+        <x:v>要確認</x:v>
+      </x:c>
+      <x:c r="E38" s="24" t="str">
+        <x:v>9N506。付属2/exam_item_masterでOID確認済み、コード値一覧は別途確認</x:v>
+      </x:c>
+      <x:c r="F38" s="21"/>
+      <x:c r="G38" s="21"/>
+      <x:c r="H38" s="21"/>
+      <x:c r="I38" s="21"/>
+      <x:c r="J38" s="21"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="24" t="str">
+        <x:v>1.2.392.200119.6.2100</x:v>
+      </x:c>
+      <x:c r="B39" s="24" t="str">
+        <x:v>陰性陽性</x:v>
+      </x:c>
+      <x:c r="C39" s="24" t="str">
+        <x:v>1/2等</x:v>
+      </x:c>
+      <x:c r="D39" s="24" t="str">
+        <x:v>陰性/陽性等</x:v>
+      </x:c>
+      <x:c r="E39" s="24" t="str">
+        <x:v>便潜血など。項目ごとの正式表示は要確認</x:v>
+      </x:c>
+      <x:c r="F39" s="21"/>
+      <x:c r="G39" s="21"/>
+      <x:c r="H39" s="21"/>
+      <x:c r="I39" s="21"/>
+      <x:c r="J39" s="21"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>